<commit_message>
update the Typo, and add todo
</commit_message>
<xml_diff>
--- a/project1/Typo.xlsx
+++ b/project1/Typo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\projects\Info_3171_group_project\project1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648FFFDE-1680-4557-B739-B351BC4CAE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2512EB5D-4FA5-4EB6-BEFA-B294C2809F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19000" yWindow="-15680" windowWidth="14010" windowHeight="12740" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
+    <workbookView xWindow="15860" yWindow="-19650" windowWidth="13830" windowHeight="18280" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Typo" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="79">
   <si>
     <t>Command TV Typography UI Pattern Library</t>
   </si>
@@ -258,6 +258,21 @@
   </si>
   <si>
     <t>6. Hierarchy: Clear distinction between titles, charts, menus, and body text</t>
+  </si>
+  <si>
+    <t>chart heading</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>chart X,Y axis and ticks color</t>
+  </si>
+  <si>
+    <t>chart X,Y ticks label</t>
+  </si>
+  <si>
+    <t>primary color</t>
   </si>
 </sst>
 </file>
@@ -296,7 +311,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -306,6 +321,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF6B5FBF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -322,12 +343,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -611,27 +633,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7653DAE9-72C2-47D7-AAA3-903529B7CD1B}">
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="25.734375" customWidth="1"/>
+    <col min="1" max="1" width="37.734375" customWidth="1"/>
     <col min="2" max="2" width="31.5234375" customWidth="1"/>
     <col min="3" max="3" width="14.26171875" customWidth="1"/>
     <col min="5" max="5" width="16.5234375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="25.8" x14ac:dyDescent="0.95">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
     </row>
     <row r="2" spans="1:11" ht="20.5" customHeight="1" x14ac:dyDescent="0.85">
       <c r="A2" s="1"/>
@@ -1258,19 +1280,27 @@
       <c r="K41" s="2"/>
     </row>
     <row r="42" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A42" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
+      <c r="A42" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C42" s="3">
+        <v>700</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
     </row>
     <row r="43" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A43" s="2"/>
@@ -1286,13 +1316,15 @@
       <c r="K43" s="2"/>
     </row>
     <row r="44" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A44" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="A44" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -1301,11 +1333,15 @@
       <c r="K44" s="2"/>
     </row>
     <row r="45" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
+      <c r="A45" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
@@ -1314,9 +1350,7 @@
       <c r="K45" s="2"/>
     </row>
     <row r="46" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A46" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -1329,7 +1363,9 @@
       <c r="K46" s="2"/>
     </row>
     <row r="47" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A47" s="2"/>
+      <c r="A47" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -1342,9 +1378,7 @@
       <c r="K47" s="2"/>
     </row>
     <row r="48" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A48" s="2" t="s">
-        <v>43</v>
-      </c>
+      <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -1357,7 +1391,9 @@
       <c r="K48" s="2"/>
     </row>
     <row r="49" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A49" s="2"/>
+      <c r="A49" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -1370,21 +1406,11 @@
       <c r="K49" s="2"/>
     </row>
     <row r="50" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
@@ -1394,20 +1420,12 @@
     </row>
     <row r="51" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A51" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C51" s="2">
-        <v>400</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>26</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
@@ -1416,21 +1434,11 @@
       <c r="K51" s="2"/>
     </row>
     <row r="52" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A52" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C52" s="2">
-        <v>500</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
@@ -1440,20 +1448,12 @@
     </row>
     <row r="53" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A53" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C53" s="2">
-        <v>400</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>49</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
@@ -1476,12 +1476,20 @@
     </row>
     <row r="55" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A55" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
@@ -1490,11 +1498,21 @@
       <c r="K55" s="2"/>
     </row>
     <row r="56" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
+      <c r="A56" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C56" s="2">
+        <v>400</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -1504,12 +1522,20 @@
     </row>
     <row r="57" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A57" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C57" s="2">
+        <v>500</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
@@ -1518,11 +1544,21 @@
       <c r="K57" s="2"/>
     </row>
     <row r="58" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
+      <c r="A58" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C58" s="2">
+        <v>400</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
@@ -1531,9 +1567,7 @@
       <c r="K58" s="2"/>
     </row>
     <row r="59" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A59" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
@@ -1546,7 +1580,9 @@
       <c r="K59" s="2"/>
     </row>
     <row r="60" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A60" s="2"/>
+      <c r="A60" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
@@ -1559,9 +1595,7 @@
       <c r="K60" s="2"/>
     </row>
     <row r="61" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A61" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -1574,7 +1608,9 @@
       <c r="K61" s="2"/>
     </row>
     <row r="62" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A62" s="2"/>
+      <c r="A62" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -1587,9 +1623,7 @@
       <c r="K62" s="2"/>
     </row>
     <row r="63" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A63" s="2" t="s">
-        <v>54</v>
-      </c>
+      <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
@@ -1602,7 +1636,9 @@
       <c r="K63" s="2"/>
     </row>
     <row r="64" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A64" s="2"/>
+      <c r="A64" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -1615,9 +1651,7 @@
       <c r="K64" s="2"/>
     </row>
     <row r="65" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A65" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -1630,7 +1664,9 @@
       <c r="K65" s="2"/>
     </row>
     <row r="66" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A66" s="2"/>
+      <c r="A66" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
@@ -1643,9 +1679,7 @@
       <c r="K66" s="2"/>
     </row>
     <row r="67" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A67" s="2" t="s">
-        <v>56</v>
-      </c>
+      <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -1658,7 +1692,9 @@
       <c r="K67" s="2"/>
     </row>
     <row r="68" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A68" s="2"/>
+      <c r="A68" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
@@ -1671,21 +1707,11 @@
       <c r="K68" s="2"/>
     </row>
     <row r="69" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A69" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
@@ -1695,20 +1721,12 @@
     </row>
     <row r="70" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A70" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C70" s="2">
-        <v>400</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>23</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
@@ -1717,21 +1735,11 @@
       <c r="K70" s="2"/>
     </row>
     <row r="71" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A71" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C71" s="2">
-        <v>400</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
@@ -1741,20 +1749,12 @@
     </row>
     <row r="72" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A72" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C72" s="2">
-        <v>500</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>23</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+      <c r="E72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -1777,12 +1777,20 @@
     </row>
     <row r="74" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A74" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
@@ -1791,11 +1799,21 @@
       <c r="K74" s="2"/>
     </row>
     <row r="75" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
+      <c r="A75" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C75" s="2">
+        <v>400</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
@@ -1805,12 +1823,20 @@
     </row>
     <row r="76" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A76" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
+        <v>59</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C76" s="2">
+        <v>400</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
@@ -1819,11 +1845,21 @@
       <c r="K76" s="2"/>
     </row>
     <row r="77" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
+      <c r="A77" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C77" s="2">
+        <v>500</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
@@ -1832,9 +1868,7 @@
       <c r="K77" s="2"/>
     </row>
     <row r="78" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A78" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
@@ -1847,7 +1881,9 @@
       <c r="K78" s="2"/>
     </row>
     <row r="79" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A79" s="2"/>
+      <c r="A79" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
@@ -1860,9 +1896,7 @@
       <c r="K79" s="2"/>
     </row>
     <row r="80" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A80" s="2" t="s">
-        <v>63</v>
-      </c>
+      <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -1875,7 +1909,9 @@
       <c r="K80" s="2"/>
     </row>
     <row r="81" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A81" s="2"/>
+      <c r="A81" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
@@ -1888,9 +1924,7 @@
       <c r="K81" s="2"/>
     </row>
     <row r="82" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A82" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
@@ -1903,7 +1937,9 @@
       <c r="K82" s="2"/>
     </row>
     <row r="83" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A83" s="2"/>
+      <c r="A83" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
@@ -1916,9 +1952,7 @@
       <c r="K83" s="2"/>
     </row>
     <row r="84" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A84" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
@@ -1931,7 +1965,9 @@
       <c r="K84" s="2"/>
     </row>
     <row r="85" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A85" s="2"/>
+      <c r="A85" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
@@ -1944,9 +1980,7 @@
       <c r="K85" s="2"/>
     </row>
     <row r="86" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A86" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
@@ -1959,7 +1993,9 @@
       <c r="K86" s="2"/>
     </row>
     <row r="87" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A87" s="2"/>
+      <c r="A87" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
@@ -1972,9 +2008,7 @@
       <c r="K87" s="2"/>
     </row>
     <row r="88" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A88" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
@@ -1987,7 +2021,9 @@
       <c r="K88" s="2"/>
     </row>
     <row r="89" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A89" s="2"/>
+      <c r="A89" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
@@ -2000,9 +2036,7 @@
       <c r="K89" s="2"/>
     </row>
     <row r="90" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A90" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
@@ -2015,7 +2049,9 @@
       <c r="K90" s="2"/>
     </row>
     <row r="91" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A91" s="2"/>
+      <c r="A91" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
@@ -2028,9 +2064,8 @@
       <c r="K91" s="2"/>
     </row>
     <row r="92" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A92" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
@@ -2042,7 +2077,9 @@
       <c r="K92" s="2"/>
     </row>
     <row r="93" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A93" s="2"/>
+      <c r="A93" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
@@ -2055,9 +2092,7 @@
       <c r="K93" s="2"/>
     </row>
     <row r="94" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A94" s="2" t="s">
-        <v>70</v>
-      </c>
+      <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
@@ -2070,7 +2105,9 @@
       <c r="K94" s="2"/>
     </row>
     <row r="95" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A95" s="2"/>
+      <c r="A95" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
@@ -2083,9 +2120,7 @@
       <c r="K95" s="2"/>
     </row>
     <row r="96" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A96" s="2" t="s">
-        <v>71</v>
-      </c>
+      <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
@@ -2098,8 +2133,9 @@
       <c r="K96" s="2"/>
     </row>
     <row r="97" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
+      <c r="A97" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
@@ -2111,9 +2147,7 @@
       <c r="K97" s="2"/>
     </row>
     <row r="98" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A98" s="2" t="s">
-        <v>72</v>
-      </c>
+      <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
@@ -2126,7 +2160,9 @@
       <c r="K98" s="2"/>
     </row>
     <row r="99" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A99" s="2"/>
+      <c r="A99" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
@@ -2139,9 +2175,7 @@
       <c r="K99" s="2"/>
     </row>
     <row r="100" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A100" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
@@ -2154,7 +2188,9 @@
       <c r="K100" s="2"/>
     </row>
     <row r="101" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A101" s="2"/>
+      <c r="A101" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
       <c r="D101" s="2"/>
@@ -2180,7 +2216,9 @@
       <c r="K102" s="2"/>
     </row>
     <row r="103" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A103" s="2"/>
+      <c r="A103" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
       <c r="D103" s="2"/>
@@ -2206,7 +2244,9 @@
       <c r="K104" s="2"/>
     </row>
     <row r="105" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A105" s="2"/>
+      <c r="A105" s="2" t="s">
+        <v>73</v>
+      </c>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
       <c r="D105" s="2"/>
@@ -2257,6 +2297,71 @@
       <c r="J108" s="2"/>
       <c r="K108" s="2"/>
     </row>
+    <row r="109" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
+      <c r="A109" s="2"/>
+      <c r="B109" s="2"/>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2"/>
+      <c r="E109" s="2"/>
+      <c r="F109" s="2"/>
+      <c r="G109" s="2"/>
+      <c r="H109" s="2"/>
+      <c r="I109" s="2"/>
+      <c r="J109" s="2"/>
+      <c r="K109" s="2"/>
+    </row>
+    <row r="110" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
+      <c r="A110" s="2"/>
+      <c r="B110" s="2"/>
+      <c r="C110" s="2"/>
+      <c r="D110" s="2"/>
+      <c r="E110" s="2"/>
+      <c r="F110" s="2"/>
+      <c r="G110" s="2"/>
+      <c r="H110" s="2"/>
+      <c r="I110" s="2"/>
+      <c r="J110" s="2"/>
+      <c r="K110" s="2"/>
+    </row>
+    <row r="111" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
+      <c r="A111" s="2"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
+      <c r="E111" s="2"/>
+      <c r="F111" s="2"/>
+      <c r="G111" s="2"/>
+      <c r="H111" s="2"/>
+      <c r="I111" s="2"/>
+      <c r="J111" s="2"/>
+      <c r="K111" s="2"/>
+    </row>
+    <row r="112" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
+      <c r="A112" s="2"/>
+      <c r="B112" s="2"/>
+      <c r="C112" s="2"/>
+      <c r="D112" s="2"/>
+      <c r="E112" s="2"/>
+      <c r="F112" s="2"/>
+      <c r="G112" s="2"/>
+      <c r="H112" s="2"/>
+      <c r="I112" s="2"/>
+      <c r="J112" s="2"/>
+      <c r="K112" s="2"/>
+    </row>
+    <row r="113" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
+      <c r="A113" s="2"/>
+      <c r="B113" s="2"/>
+      <c r="C113" s="2"/>
+      <c r="D113" s="2"/>
+      <c r="E113" s="2"/>
+      <c r="F113" s="2"/>
+      <c r="G113" s="2"/>
+      <c r="H113" s="2"/>
+      <c r="I113" s="2"/>
+      <c r="J113" s="2"/>
+      <c r="K113" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
feat: update font styles in charts to use Merriweather and adjust weight for consistency
</commit_message>
<xml_diff>
--- a/project1/Typo.xlsx
+++ b/project1/Typo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2512EB5D-4FA5-4EB6-BEFA-B294C2809F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D0A5A7-C5BE-483C-906B-20AEF54D68F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15860" yWindow="-19650" windowWidth="13830" windowHeight="18280" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
+    <workbookView xWindow="11442" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Typo" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="81">
   <si>
     <t>Command TV Typography UI Pattern Library</t>
   </si>
@@ -272,7 +272,13 @@
     <t>chart X,Y ticks label</t>
   </si>
   <si>
-    <t>primary color</t>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">secondary color #8d1179 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">secondary  color #8d1179 </t>
   </si>
 </sst>
 </file>
@@ -1320,10 +1326,12 @@
         <v>76</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
+      <c r="D44" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="E44" s="3"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -1337,10 +1345,12 @@
         <v>77</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
+      <c r="D45" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="E45" s="3"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
@@ -1463,7 +1473,9 @@
     </row>
     <row r="54" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
+      <c r="B54" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -1498,22 +1510,22 @@
       <c r="K55" s="2"/>
     </row>
     <row r="56" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A56" s="2" t="s">
+      <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C56" s="2">
-        <v>400</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E56" s="2" t="s">
+      <c r="C56" s="3">
+        <v>700</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F56" s="2"/>
+      <c r="F56" s="3"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -1521,22 +1533,22 @@
       <c r="K56" s="2"/>
     </row>
     <row r="57" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A57" s="2" t="s">
+      <c r="A57" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C57" s="3">
         <v>500</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="D57" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E57" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F57" s="2"/>
+      <c r="F57" s="3"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -1544,22 +1556,22 @@
       <c r="K57" s="2"/>
     </row>
     <row r="58" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
-      <c r="A58" s="2" t="s">
+      <c r="A58" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C58" s="3">
         <v>400</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D58" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E58" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F58" s="2"/>
+      <c r="F58" s="3"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>

</xml_diff>

<commit_message>
feat: update text colors in charts to improve visibility and consistency
</commit_message>
<xml_diff>
--- a/project1/Typo.xlsx
+++ b/project1/Typo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D0A5A7-C5BE-483C-906B-20AEF54D68F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBED6426-74DC-49DC-9496-9F8375BDDE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11442" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
+    <workbookView xWindow="12720" yWindow="0" windowWidth="10398" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Typo" sheetId="1" r:id="rId1"/>
@@ -275,10 +275,10 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">secondary color #8d1179 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">secondary  color #8d1179 </t>
+    <t>primary color #3b118d</t>
+  </si>
+  <si>
+    <t>primary  color #3b118d</t>
   </si>
 </sst>
 </file>
@@ -2379,5 +2379,6 @@
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adjust chart positioning and update styles for improved readability and consistency
</commit_message>
<xml_diff>
--- a/project1/Typo.xlsx
+++ b/project1/Typo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBED6426-74DC-49DC-9496-9F8375BDDE7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE39B51-A86E-4AD2-B5C4-DD273C888B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12720" yWindow="0" windowWidth="10398" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
+    <workbookView xWindow="12588" yWindow="0" windowWidth="10530" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Typo" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="82">
   <si>
     <t>Command TV Typography UI Pattern Library</t>
   </si>
@@ -272,13 +272,16 @@
     <t>chart X,Y ticks label</t>
   </si>
   <si>
+    <t>primary color</t>
+  </si>
+  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>primary color #3b118d</t>
-  </si>
-  <si>
-    <t>primary  color #3b118d</t>
+    <t xml:space="preserve">secondary color #8d1179 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">secondary  color #8d1179 </t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1329,7 @@
         <v>76</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3" t="s">
@@ -1345,7 +1348,7 @@
         <v>77</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3" t="s">
@@ -1474,7 +1477,7 @@
     <row r="54" spans="1:11" ht="23.1" x14ac:dyDescent="0.85">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
@@ -1525,7 +1528,9 @@
       <c r="E56" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F56" s="3"/>
+      <c r="F56" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>

</xml_diff>